<commit_message>
Polish Kotak header nav: mega-menu two-panel, simple dropdowns, icons
- Mega menus (Personal/Business/NRI): two-panel layout (sidebar + vertical
  link column), "Discover {X}" heading, product icons, viewport-centered.
- Simple menus (About Us/Learn/Help): single link list with first item as a
  white rounded card, no sidebar.
- Top-level items: dropdown chevron + red active underline on <p> labels.
- Brand logo image; closed-on-load; product/category SVG icons in /icons.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,22 +37,37 @@
     <t>url</t>
   </si>
   <si>
+    <t>forex-card.report.json</t>
+  </si>
+  <si>
+    <t>["hero-p"]</t>
+  </si>
+  <si>
+    <t>forex-card</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-08-11T11:18:55.155Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://www.kotak.bank.in/en/personal-banking/cards/prepaid-card/forex-card.html</t>
+  </si>
+  <si>
     <t>nav.report.json</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>nav</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>nav-fragment</t>
   </si>
   <si>
-    <t>2026-08-13T10:35:17.461Z</t>
+    <t>2026-08-14T08:46:48.756Z</t>
   </si>
   <si>
     <t>http://localhost:3000/nav</t>
@@ -480,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -489,7 +504,7 @@
     <col min="5" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="46" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -532,13 +547,13 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
       </c>
       <c r="H2" t="s">
         <v>14</v>
@@ -549,10 +564,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -564,36 +579,62 @@
         <v>18</v>
       </c>
       <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" t="s">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>